<commit_message>
Carga masiva de stock productos sucursal
</commit_message>
<xml_diff>
--- a/public/files/formato_producto_sucursals.xlsx
+++ b/public/files/formato_producto_sucursals.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5688"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="13">
   <si>
     <t/>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>CÓDIGO*</t>
+  </si>
+  <si>
+    <t>STOCK</t>
   </si>
 </sst>
 </file>
@@ -444,7 +447,7 @@
     <col min="7" max="9" width="8.3984375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.69921875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.3984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7" customWidth="1"/>
     <col min="13" max="13" width="9.3984375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.5" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="9.69921875" bestFit="1" customWidth="1"/>
@@ -487,6 +490,9 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">

</xml_diff>